<commit_message>
Actualizar pipeline y datos: split Flex/pasante, Gastos de Agencia, costos corregidos
- build_pnl_data.py/build_dashboard_data.py/build_sheet.py: split de envio Flex
  real vs pasante Full/Colecta (ingreso/egreso), nueva categoria "Gastos de
  Agencia" como costo fijo, PERIODOS actualizado hasta septiembre parcial (13/9)
- data/Costos.xlsx: correcciones de costos (Treonato, Creatina, Bisglicinato,
  Toalla de cara, Cuchillo Postre Nicols x6) + altos SKUs faltantes
- base_*.json, dashboard_data/output, ordenes_*.json: datos regenerados con
  el pipeline al 14/9
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="D43" s="0" t="n">
-        <v>6474.98</v>
+        <v>7834.73</v>
       </c>
       <c r="E43" s="8" t="n">
         <v>46237</v>
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="D44" s="0" t="n">
-        <v>7063.45</v>
+        <v>8546.77</v>
       </c>
       <c r="E44" s="8" t="n">
         <v>46237</v>
@@ -1468,30 +1468,303 @@
         </is>
       </c>
       <c r="D53" s="0" t="n">
-        <v>1454.55</v>
+        <v>1760</v>
       </c>
       <c r="E53" s="8" t="n">
         <v>46143</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="0" t="n">
         <v>50030</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="0" t="inlineStr">
         <is>
           <t>MLA1977669679</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="0" t="inlineStr">
         <is>
           <t>Creatina En Pote Star Nutrition 300 Gr Monohidrato Micronizado</t>
         </is>
       </c>
-      <c r="D54" t="n">
-        <v>12909.64</v>
+      <c r="D54" s="0" t="n">
+        <v>15620.66</v>
       </c>
       <c r="E54" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="n">
+        <v>50033</v>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>MLA1977869383</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>Geonat Aceite De Pescado Omega 3 Omeganat Colesterol 60 Capsulas Sin Sabor</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="n">
+        <v>11229.81</v>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="n">
+        <v>50033</v>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>MLA1977869381</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t>Omega 3 Epa Aceite Pescado Geonat Colesterol 60 Capsulas Sin Sabor</t>
+        </is>
+      </c>
+      <c r="D56" s="0" t="n">
+        <v>11229.81</v>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="n">
+        <v>50005</v>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>MLA1939972297</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>Toallon Oregon Hotelero 550gr 90x150 Plus (var. 2)</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="n">
+        <v>12656</v>
+      </c>
+      <c r="E57" s="8" t="n">
+        <v>46224</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="n">
+        <v>50030</v>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>MLA1977669677</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato Star Nutrition Micronizada 300g Neutro (var.)</t>
+        </is>
+      </c>
+      <c r="D58" s="0" t="n">
+        <v>15620.66</v>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="n">
+        <v>50014</v>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>MLA1947819693</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>L-arginina + L-citrulina + Ginseng M1 Energy (var.)</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="n">
+        <v>8239.33</v>
+      </c>
+      <c r="E59" s="8" t="n">
+        <v>46224</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="n">
+        <v>50029</v>
+      </c>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t>MLA3770705240</t>
+        </is>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato Ena Sport 300g Micronizada 60 Servicios Sin Sabor</t>
+        </is>
+      </c>
+      <c r="D60" s="0" t="n">
+        <v>15829.26</v>
+      </c>
+      <c r="E60" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="n">
+        <v>50032</v>
+      </c>
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t>MLA1977868561</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>Colageno Hidrolizado Star Nutrition Pote 210g Limon</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="n">
+        <v>10470.6</v>
+      </c>
+      <c r="E61" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="n">
+        <v>50032</v>
+      </c>
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t>MLA1977868557</t>
+        </is>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t>Colageno Hidrolizado Star Nutrition Pote 210g Limon</t>
+        </is>
+      </c>
+      <c r="D62" s="0" t="n">
+        <v>10470.6</v>
+      </c>
+      <c r="E62" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="n">
+        <v>10007</v>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t>MLA2275436422</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t>Cuchillo Postre Nicols Corintia Inox Pulido Brillante X6</t>
+        </is>
+      </c>
+      <c r="D63" s="0" t="n">
+        <v>12720</v>
+      </c>
+      <c r="E63" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="n">
+        <v>50024</v>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>MLA1961104511</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>Juego Set Toalla Toallon Oregon 630 G/m2 Ultra Blanco</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="n">
+        <v>28888</v>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="n">
+        <v>50025</v>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>MLA1961104507</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>Juego Set Toalla Toallon Oregon 630 G/m2 Ultra Gris Oscuro Aluminium</t>
+        </is>
+      </c>
+      <c r="D65" s="0" t="n">
+        <v>28888</v>
+      </c>
+      <c r="E65" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="n">
+        <v>50026</v>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t>MLA1961117287</t>
+        </is>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t>Juego Set Toalla Toallon Oregon 630 G/m2 Ultra Marron Oscuro Wood</t>
+        </is>
+      </c>
+      <c r="D66" s="0" t="n">
+        <v>28888</v>
+      </c>
+      <c r="E66" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="n">
+        <v>50027</v>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t>MLA1961104509</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>Juego Set Toalla Toallon Oregon 630 G/m2 Ultra Marron Claro Honey</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="n">
+        <v>28888</v>
+      </c>
+      <c r="E67" s="8" t="n">
         <v>46143</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corregir costo faltante de SKU 50029 (item republicado)
La orden 2000018475229818 (2026-09-15) mostraba margen de 68% porque
el item MLA3770867494 (republicacion de la misma creatina, SKU 50029)
no tenia costo cargado en data/Costos.xlsx -- el lookup es por item_id
y ese id nuevo no estaba, asi que cayo a $0 en vez de avisar.

Se agrega el mismo costo del item viejo (MLA3770705240, $15.829,26
sin IVA), confirmado por Lucas. Margen real de esa orden: 4,52% (antes
68,37%). Recalculado base_ventas/pnl/dashboard para esa orden y subido.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fCWZQxxkHvBtayzxg2duj
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -1768,6 +1768,27 @@
         <v>46143</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>50029</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>MLA3770867494</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Creatina Monohidratada Ena Sport Micronizada 300g Neutro Neutro</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>15829.26</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corregir costo faltante de Creatina Ena Sport (SKU 50029, item_id nuevo)
MercadoLibre recreo la publicacion de la Creatina Monohidratada Ena
Sport 300g bajo un item_id nuevo (MLA3770867494) a partir del 15/09;
el item_id viejo (MLA3770705240) dejo de vender el 09/09. Costos.xlsx
solo tenia el costo mapeado contra el item_id viejo, asi que las 3
ordenes del item_id nuevo (15-16/09) quedaron con costo $0 en
base_ventas. Se agrega el mismo costo vigente ($15.829,26 s/IVA) contra
el item_id nuevo y se recalculan esas 3 ordenes -- COGS de septiembre
sube $57.460,20 (3 x $19.153,40 c/IVA).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -1768,6 +1768,27 @@
         <v>46143</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>50029</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>MLA3770867494</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Creatina Monohidratada Ena Sport Micronizada 300g Neutro Neutro</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>15829.26</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar costo de reposicion de toallas Oregon (vigente 8/9) y agregar chequeo diario de productos sin costo
Toalla de Mano 550 (SKU 50004): 4448 -> 4704 s/IVA
Toalla de Cara 400 (SKU 50028): 1760 -> 1856 s/IVA (sin ventas en el rango afectado)
Toallon 550 (SKU 50005): 12656 -> 13328 s/IVA

Costo de Reposicion: se agregan filas nuevas en data/Costos.xlsx con fecha
2026-09-08 (no se pisan las anteriores), y se recalcula costo_s/costo_c y
resultado neto/margen solo para las 3 ordenes de base_ventas.json de esos
productos vendidas desde esa fecha -- las anteriores quedan con el costo
viejo. P&L/dashboard/Sheet regenerados y dashboard republicado.

Se agrega check_productos_sin_costo.py (pedido de Lucas) que compara la foto
mas reciente de stock_valorizado contra data/Costos.xlsx y lista que
publicaciones activas no tienen costo cargado -- ahora forma parte del
pipeline de actualizar-tablero (Paso 7.5), para que se chequee a diario.
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -1769,24 +1769,150 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="n">
+      <c r="A68" s="0" t="n">
         <v>50029</v>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="0" t="inlineStr">
         <is>
           <t>MLA3770867494</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="0" t="inlineStr">
         <is>
           <t>Creatina Monohidratada Ena Sport Micronizada 300g Neutro Neutro</t>
         </is>
       </c>
-      <c r="D68" t="n">
+      <c r="D68" s="0" t="n">
         <v>15829.26</v>
       </c>
       <c r="E68" s="8" t="n">
         <v>46143</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>50004</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>MLA3232809762</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Toalla Oregon Hotelera 550gr 45x80 Plus</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>4704</v>
+      </c>
+      <c r="E69" s="8" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>50004</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>MLA3571928900</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Toalla Oregon Hotelera 550gr 45x80 Plus (var.)</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>4704</v>
+      </c>
+      <c r="E70" s="8" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>50028</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>MLA1961130867</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Toalla De Cara Facial Oregon Hotelera 100% Algodon 400gr Blanca</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>1856</v>
+      </c>
+      <c r="E71" s="8" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>50005</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>MLA3232759300</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Toallon Oregon Hotelero 550gr 90x150 Plus</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>13328</v>
+      </c>
+      <c r="E72" s="8" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>50005</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>MLA3566784906</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Toallon Oregon Hotelero 550gr 90x150 Plus (var.)</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>13328</v>
+      </c>
+      <c r="E73" s="8" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>50005</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>MLA1939972297</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Toallon Oregon Hotelero 550gr 90x150 Plus (var. 2)</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>13328</v>
+      </c>
+      <c r="E74" s="8" t="n">
+        <v>46273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cargar costo de los 10 productos activos que no tenian ninguno
Cuchillo Mesa Nicols Delta (20006), Cuchillo Grille Nicols Corintia (10009),
Whey Protein Gold Nutrition Vainilla/Chocolate (50039/50040), Tabla de Picar
(50001), Kit x3 Toalla Cara (50028), Cuchara Postre Nicols Corintia (10003),
Cuchillo Mesa Nicols Corintia (10006), Untador Nicols Atlas (30009), Tenedor
Postre Nicols Corintia (10001) -- costos pasados por Lucas, cargados en
data/Costos.xlsx con fecha 2026-05-01 (retroactivo, pedido explicito de
Lucas) para que cubra tambien las 7 ordenes de Whey Protein ya vendidas
(19-21/9) que habian quedado con costo $0 y margen inflado.

check_productos_sin_costo.py confirma que ya no queda ninguna publicacion
activa sin costo. P&L y dashboard regenerados y republicados; el Sheet de
Google quedo pendiente porque el token OAuth esta revocado (ver auth_google.py).
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -1790,20 +1790,20 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="n">
+      <c r="A69" s="0" t="n">
         <v>50004</v>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="0" t="inlineStr">
         <is>
           <t>MLA3232809762</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="0" t="inlineStr">
         <is>
           <t>Toalla Oregon Hotelera 550gr 45x80 Plus</t>
         </is>
       </c>
-      <c r="D69" t="n">
+      <c r="D69" s="0" t="n">
         <v>4704</v>
       </c>
       <c r="E69" s="8" t="n">
@@ -1811,20 +1811,20 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="n">
+      <c r="A70" s="0" t="n">
         <v>50004</v>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="0" t="inlineStr">
         <is>
           <t>MLA3571928900</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="0" t="inlineStr">
         <is>
           <t>Toalla Oregon Hotelera 550gr 45x80 Plus (var.)</t>
         </is>
       </c>
-      <c r="D70" t="n">
+      <c r="D70" s="0" t="n">
         <v>4704</v>
       </c>
       <c r="E70" s="8" t="n">
@@ -1832,20 +1832,20 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="n">
+      <c r="A71" s="0" t="n">
         <v>50028</v>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="0" t="inlineStr">
         <is>
           <t>MLA1961130867</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="0" t="inlineStr">
         <is>
           <t>Toalla De Cara Facial Oregon Hotelera 100% Algodon 400gr Blanca</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D71" s="0" t="n">
         <v>1856</v>
       </c>
       <c r="E71" s="8" t="n">
@@ -1853,20 +1853,20 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="n">
+      <c r="A72" s="0" t="n">
         <v>50005</v>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="0" t="inlineStr">
         <is>
           <t>MLA3232759300</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="0" t="inlineStr">
         <is>
           <t>Toallon Oregon Hotelero 550gr 90x150 Plus</t>
         </is>
       </c>
-      <c r="D72" t="n">
+      <c r="D72" s="0" t="n">
         <v>13328</v>
       </c>
       <c r="E72" s="8" t="n">
@@ -1874,20 +1874,20 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="n">
+      <c r="A73" s="0" t="n">
         <v>50005</v>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="0" t="inlineStr">
         <is>
           <t>MLA3566784906</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="0" t="inlineStr">
         <is>
           <t>Toallon Oregon Hotelero 550gr 90x150 Plus (var.)</t>
         </is>
       </c>
-      <c r="D73" t="n">
+      <c r="D73" s="0" t="n">
         <v>13328</v>
       </c>
       <c r="E73" s="8" t="n">
@@ -1895,24 +1895,234 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="n">
+      <c r="A74" s="0" t="n">
         <v>50005</v>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="0" t="inlineStr">
         <is>
           <t>MLA1939972297</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="0" t="inlineStr">
         <is>
           <t>Toallon Oregon Hotelero 550gr 90x150 Plus (var. 2)</t>
         </is>
       </c>
-      <c r="D74" t="n">
+      <c r="D74" s="0" t="n">
         <v>13328</v>
       </c>
       <c r="E74" s="8" t="n">
         <v>46273</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>20006</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>MLA2275448906</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Cuchillo Mesa Nicols Delta x6</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>28543.87</v>
+      </c>
+      <c r="E75" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>10009</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MLA2275436420</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Cuchillo Grille Nicols Corintia x6</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>19471.2</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>50039</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>MLA2090594323</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Whey Protein Gold Nutrition 2Lb Vainilla</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>48408.07</v>
+      </c>
+      <c r="E77" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>50040</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>MLA3949765754</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Whey Protein Gold Nutrition 2Lb Chocolate</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>48408.07</v>
+      </c>
+      <c r="E78" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>50001</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>MLA1729211787</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Tabla De Picar 35x24cm</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E79" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>50028</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>MLA2091401039</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Kit X 3 Toalla Cara Oregon 30x50</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>5568</v>
+      </c>
+      <c r="E80" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>10003</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>MLA1516293305</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Cuchara Postre Nicols Corintia x6</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>8238.799999999999</v>
+      </c>
+      <c r="E81" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>10006</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MLA1516301921</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Cuchillo Mesa Nicols Corintia x6</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>14982.24</v>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>30009</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MLA2275436424</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Untador Nicols Atlas x6</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>7759.29</v>
+      </c>
+      <c r="E83" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>10001</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MLA2275397446</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Tenedor Postre Nicols Corintia x6</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>8238.799999999999</v>
+      </c>
+      <c r="E84" s="8" t="n">
+        <v>46143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cargar costo de Mate Imperial (negro/marron) y del item nuevo del Kit x3 Toallas
- Mate Imperial SKU 50041/50042: 21.900 s/IVA
- Kit x3 Toalla Cara SKU 50028: el costo estaba cargado solo para
  MLA2091401039, pero la publicacion activa es MLA2091401043 -- se agrega
  ese item_id con el mismo costo (5.568 s/IVA)
- Recalculada la orden 2000018581082790 (21/09, 4 kits) que habia quedado
  con costo $0; P&L/dashboard/Sheet regenerados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SUg2PMsfSxbYhkWoikRK5a
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -1916,20 +1916,20 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="n">
+      <c r="A75" s="0" t="n">
         <v>20006</v>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="0" t="inlineStr">
         <is>
           <t>MLA2275448906</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="0" t="inlineStr">
         <is>
           <t>Cuchillo Mesa Nicols Delta x6</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D75" s="0" t="n">
         <v>28543.87</v>
       </c>
       <c r="E75" s="8" t="n">
@@ -1937,20 +1937,20 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="n">
+      <c r="A76" s="0" t="n">
         <v>10009</v>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="0" t="inlineStr">
         <is>
           <t>MLA2275436420</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="0" t="inlineStr">
         <is>
           <t>Cuchillo Grille Nicols Corintia x6</t>
         </is>
       </c>
-      <c r="D76" t="n">
+      <c r="D76" s="0" t="n">
         <v>19471.2</v>
       </c>
       <c r="E76" s="8" t="n">
@@ -1958,20 +1958,20 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="n">
+      <c r="A77" s="0" t="n">
         <v>50039</v>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="0" t="inlineStr">
         <is>
           <t>MLA2090594323</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="0" t="inlineStr">
         <is>
           <t>Whey Protein Gold Nutrition 2Lb Vainilla</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D77" s="0" t="n">
         <v>48408.07</v>
       </c>
       <c r="E77" s="8" t="n">
@@ -1979,20 +1979,20 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="n">
+      <c r="A78" s="0" t="n">
         <v>50040</v>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="0" t="inlineStr">
         <is>
           <t>MLA3949765754</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="0" t="inlineStr">
         <is>
           <t>Whey Protein Gold Nutrition 2Lb Chocolate</t>
         </is>
       </c>
-      <c r="D78" t="n">
+      <c r="D78" s="0" t="n">
         <v>48408.07</v>
       </c>
       <c r="E78" s="8" t="n">
@@ -2000,20 +2000,20 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="n">
+      <c r="A79" s="0" t="n">
         <v>50001</v>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="0" t="inlineStr">
         <is>
           <t>MLA1729211787</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="0" t="inlineStr">
         <is>
           <t>Tabla De Picar 35x24cm</t>
         </is>
       </c>
-      <c r="D79" t="n">
+      <c r="D79" s="0" t="n">
         <v>28000</v>
       </c>
       <c r="E79" s="8" t="n">
@@ -2021,20 +2021,20 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="n">
+      <c r="A80" s="0" t="n">
         <v>50028</v>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="0" t="inlineStr">
         <is>
           <t>MLA2091401039</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="0" t="inlineStr">
         <is>
           <t>Kit X 3 Toalla Cara Oregon 30x50</t>
         </is>
       </c>
-      <c r="D80" t="n">
+      <c r="D80" s="0" t="n">
         <v>5568</v>
       </c>
       <c r="E80" s="8" t="n">
@@ -2042,20 +2042,20 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="n">
+      <c r="A81" s="0" t="n">
         <v>10003</v>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="0" t="inlineStr">
         <is>
           <t>MLA1516293305</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="0" t="inlineStr">
         <is>
           <t>Cuchara Postre Nicols Corintia x6</t>
         </is>
       </c>
-      <c r="D81" t="n">
+      <c r="D81" s="0" t="n">
         <v>8238.799999999999</v>
       </c>
       <c r="E81" s="8" t="n">
@@ -2063,20 +2063,20 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="n">
+      <c r="A82" s="0" t="n">
         <v>10006</v>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="0" t="inlineStr">
         <is>
           <t>MLA1516301921</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="0" t="inlineStr">
         <is>
           <t>Cuchillo Mesa Nicols Corintia x6</t>
         </is>
       </c>
-      <c r="D82" t="n">
+      <c r="D82" s="0" t="n">
         <v>14982.24</v>
       </c>
       <c r="E82" s="8" t="n">
@@ -2084,20 +2084,20 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="n">
+      <c r="A83" s="0" t="n">
         <v>30009</v>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="0" t="inlineStr">
         <is>
           <t>MLA2275436424</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="0" t="inlineStr">
         <is>
           <t>Untador Nicols Atlas x6</t>
         </is>
       </c>
-      <c r="D83" t="n">
+      <c r="D83" s="0" t="n">
         <v>7759.29</v>
       </c>
       <c r="E83" s="8" t="n">
@@ -2105,23 +2105,86 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="n">
+      <c r="A84" s="0" t="n">
         <v>10001</v>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="0" t="inlineStr">
         <is>
           <t>MLA2275397446</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="0" t="inlineStr">
         <is>
           <t>Tenedor Postre Nicols Corintia x6</t>
         </is>
       </c>
-      <c r="D84" t="n">
+      <c r="D84" s="0" t="n">
         <v>8238.799999999999</v>
       </c>
       <c r="E84" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>50041</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>MLA2097402363</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Mate Imperial Cuero Calabaza Con Bombilla Negro</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>21900</v>
+      </c>
+      <c r="E85" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>50042</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MLA2097402365</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Mate Imperial Cuero Calabaza Con Bombilla Marron</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>21900</v>
+      </c>
+      <c r="E86" s="8" t="n">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>50028</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>MLA2091401043</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Kit X 3 Toalla Cara Oregon 30x50 (var.)</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>5568</v>
+      </c>
+      <c r="E87" s="8" t="n">
         <v>46143</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Costo nuevo Yerba Canarias desde 08/09 y nombres de categoria faltantes
- data/Costos.xlsx: Canarias Tradicional $7.132,89 s/IVA y Serena $7.657,22 s/IVA
  vigentes desde 08/09 (todas sus publicaciones, incl. Sin Palo MLA1803968517 y
  las 2 de Serena que no tenian costo; Combo X3 = 3x Tradicional)
- base_ventas: recalculadas las 12 ordenes de yerba de septiembre (23-24/09)
- cat_names.json: MLA416552/MLA436257 -> Toallones, MLA114456 -> Botas
- cat_names.py: los builds completan solos cualquier categoria nueva con el
  nombre de /categories/{id} en vez de mostrar el ID crudo
- P&L/dashboard/Sheet regenerados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tbKEPC5GDHGx2zvRhC5JY
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -53,7 +53,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -69,6 +69,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -344,7 +345,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -2126,20 +2127,20 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="n">
+      <c r="A85" s="0" t="n">
         <v>50041</v>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="0" t="inlineStr">
         <is>
           <t>MLA2097402363</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="0" t="inlineStr">
         <is>
           <t>Mate Imperial Cuero Calabaza Con Bombilla Negro</t>
         </is>
       </c>
-      <c r="D85" t="n">
+      <c r="D85" s="0" t="n">
         <v>21900</v>
       </c>
       <c r="E85" s="8" t="n">
@@ -2147,20 +2148,20 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="n">
+      <c r="A86" s="0" t="n">
         <v>50042</v>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="0" t="inlineStr">
         <is>
           <t>MLA2097402365</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="0" t="inlineStr">
         <is>
           <t>Mate Imperial Cuero Calabaza Con Bombilla Marron</t>
         </is>
       </c>
-      <c r="D86" t="n">
+      <c r="D86" s="0" t="n">
         <v>21900</v>
       </c>
       <c r="E86" s="8" t="n">
@@ -2168,24 +2169,171 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="0" t="n">
         <v>50028</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="0" t="inlineStr">
         <is>
           <t>MLA2091401043</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="0" t="inlineStr">
         <is>
           <t>Kit X 3 Toalla Cara Oregon 30x50 (var.)</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D87" s="0" t="n">
         <v>5568</v>
       </c>
       <c r="E87" s="8" t="n">
         <v>46143</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>50006</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>MLA3283469316</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Yerba Mate Canarias Tradicional 1kg</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>7132.89</v>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>50006</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MLA3372513504</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Yerba Mate Canarias Tradicional 1kg (var.)</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>7132.89</v>
+      </c>
+      <c r="E89" s="9" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>50006</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MLA1778680761</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Yerba Mate Canarias Tradicional 1kg Sin Palo</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>7132.89</v>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>50006</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MLA1803968517</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Yerba Mate Canarias Tradicional 1kg Sin Palo (2)</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>7132.89</v>
+      </c>
+      <c r="E91" s="9" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>50006</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>MLA1805789665</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Yerba Canarias 1kg Combo X3</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>21398.67</v>
+      </c>
+      <c r="E92" s="9" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>50037</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>MLA3949953586</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Canarias Serena 1kg</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>7657.22</v>
+      </c>
+      <c r="E93" s="9" t="n">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>50037</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>MLA3949953582</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Yerba Mate Canarias Serena Compuesta Con Hierbas 1kg</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>7657.22</v>
+      </c>
+      <c r="E94" s="9" t="n">
+        <v>46273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Costo Treonato de Magnesio: 10.421 s/IVA desde 01/09
Nueva fila en data/Costos.xlsx (MLA3677881124, vigente 2026-09-01) y
recalculo de costo/resultado/margen de las 173 ordenes de septiembre en
base_ventas (224 unidades). COGS septiembre +$507.992 c/IVA.
P&L, dashboard y Sheet regenerados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gs48vNuGc4JjNeT61So13T
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -345,7 +345,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -2190,20 +2190,20 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="n">
+      <c r="A88" s="0" t="n">
         <v>50006</v>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="0" t="inlineStr">
         <is>
           <t>MLA3283469316</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="0" t="inlineStr">
         <is>
           <t>Yerba Mate Canarias Tradicional 1kg</t>
         </is>
       </c>
-      <c r="D88" t="n">
+      <c r="D88" s="0" t="n">
         <v>7132.89</v>
       </c>
       <c r="E88" s="9" t="n">
@@ -2211,20 +2211,20 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
+      <c r="A89" s="0" t="n">
         <v>50006</v>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="0" t="inlineStr">
         <is>
           <t>MLA3372513504</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="0" t="inlineStr">
         <is>
           <t>Yerba Mate Canarias Tradicional 1kg (var.)</t>
         </is>
       </c>
-      <c r="D89" t="n">
+      <c r="D89" s="0" t="n">
         <v>7132.89</v>
       </c>
       <c r="E89" s="9" t="n">
@@ -2232,20 +2232,20 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="n">
+      <c r="A90" s="0" t="n">
         <v>50006</v>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="0" t="inlineStr">
         <is>
           <t>MLA1778680761</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="0" t="inlineStr">
         <is>
           <t>Yerba Mate Canarias Tradicional 1kg Sin Palo</t>
         </is>
       </c>
-      <c r="D90" t="n">
+      <c r="D90" s="0" t="n">
         <v>7132.89</v>
       </c>
       <c r="E90" s="9" t="n">
@@ -2253,20 +2253,20 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="n">
+      <c r="A91" s="0" t="n">
         <v>50006</v>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="0" t="inlineStr">
         <is>
           <t>MLA1803968517</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="0" t="inlineStr">
         <is>
           <t>Yerba Mate Canarias Tradicional 1kg Sin Palo (2)</t>
         </is>
       </c>
-      <c r="D91" t="n">
+      <c r="D91" s="0" t="n">
         <v>7132.89</v>
       </c>
       <c r="E91" s="9" t="n">
@@ -2274,20 +2274,20 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="n">
+      <c r="A92" s="0" t="n">
         <v>50006</v>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="0" t="inlineStr">
         <is>
           <t>MLA1805789665</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="0" t="inlineStr">
         <is>
           <t>Yerba Canarias 1kg Combo X3</t>
         </is>
       </c>
-      <c r="D92" t="n">
+      <c r="D92" s="0" t="n">
         <v>21398.67</v>
       </c>
       <c r="E92" s="9" t="n">
@@ -2295,20 +2295,20 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="n">
+      <c r="A93" s="0" t="n">
         <v>50037</v>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="0" t="inlineStr">
         <is>
           <t>MLA3949953586</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="0" t="inlineStr">
         <is>
           <t>Canarias Serena 1kg</t>
         </is>
       </c>
-      <c r="D93" t="n">
+      <c r="D93" s="0" t="n">
         <v>7657.22</v>
       </c>
       <c r="E93" s="9" t="n">
@@ -2316,24 +2316,45 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="n">
+      <c r="A94" s="0" t="n">
         <v>50037</v>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="0" t="inlineStr">
         <is>
           <t>MLA3949953582</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C94" s="0" t="inlineStr">
         <is>
           <t>Yerba Mate Canarias Serena Compuesta Con Hierbas 1kg</t>
         </is>
       </c>
-      <c r="D94" t="n">
+      <c r="D94" s="0" t="n">
         <v>7657.22</v>
       </c>
       <c r="E94" s="9" t="n">
         <v>46273</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="n">
+        <v>50020</v>
+      </c>
+      <c r="B95" s="0" t="inlineStr">
+        <is>
+          <t>MLA3677881124</t>
+        </is>
+      </c>
+      <c r="C95" s="0" t="inlineStr">
+        <is>
+          <t>Treonato De Magnesio 1000 Mg Geonat Para Concentracion Y Memoria 60 Comprimidos Sin Sabor</t>
+        </is>
+      </c>
+      <c r="D95" s="0" t="n">
+        <v>10421</v>
+      </c>
+      <c r="E95" s="8" t="n">
+        <v>46266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cargar costos de Iso Gold, Whey Gold y Creatina Black Line
- data/Costos.xlsx: costos s/IVA de MLA2090592695 (55.166,94), MLA2090594295 (44.330,58) y MLA2123732493 (13.446,94)
- base_ventas: reprocesadas 3 ordenes (30/09, 01/10, 02/10) que tenian costo $0
- P&L, dashboard y Sheet regenerados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tixe6AT2wcfLTvysmThrtp
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -345,7 +345,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -2357,6 +2357,69 @@
         <v>46266</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>50038</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>MLA2090592695</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Iso Gold Protein 2lbs Gold Nutrition® Proteína Aislada Sabor Chocolate Gourmet Milk Chocolate</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>55166.94</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>50040</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>MLA2090594295</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Whey Protein Gold Nutrition 2 Libras Proteína 100% Gourmet Milk Chocolate</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>44330.58</v>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>50043</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>MLA2123732493</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Creatina Gold Nutrition Black Line En Polvo Sin Sabor X 300g</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>13446.94</v>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>46300</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cargar costos 50038/50039/50043 (+IVA /1.21) y reprocesar ordenes con costo 0
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B6Ej9HH2pZG2xD9hqQfC1p
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -345,7 +345,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="7.38" customWidth="1" style="7" min="1" max="1"/>
@@ -2358,65 +2358,149 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="n">
+      <c r="A96" s="0" t="n">
         <v>50038</v>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="0" t="inlineStr">
         <is>
           <t>MLA2090592695</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="0" t="inlineStr">
         <is>
           <t>Iso Gold Protein 2lbs Gold Nutrition® Proteína Aislada Sabor Chocolate Gourmet Milk Chocolate</t>
         </is>
       </c>
-      <c r="D96" t="n">
-        <v>55166.94</v>
+      <c r="D96" s="0" t="n">
+        <v>45592.51</v>
       </c>
       <c r="E96" s="8" t="n">
         <v>46300</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="n">
+      <c r="A97" s="0" t="n">
         <v>50040</v>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="0" t="inlineStr">
         <is>
           <t>MLA2090594295</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="0" t="inlineStr">
         <is>
           <t>Whey Protein Gold Nutrition 2 Libras Proteína 100% Gourmet Milk Chocolate</t>
         </is>
       </c>
-      <c r="D97" t="n">
-        <v>44330.58</v>
+      <c r="D97" s="0" t="n">
+        <v>36636.84</v>
       </c>
       <c r="E97" s="8" t="n">
         <v>46300</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="n">
+      <c r="A98" s="0" t="n">
         <v>50043</v>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B98" s="0" t="inlineStr">
         <is>
           <t>MLA2123732493</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" s="0" t="inlineStr">
         <is>
           <t>Creatina Gold Nutrition Black Line En Polvo Sin Sabor X 300g</t>
         </is>
       </c>
-      <c r="D98" t="n">
-        <v>13446.94</v>
+      <c r="D98" s="0" t="n">
+        <v>11113.17</v>
       </c>
       <c r="E98" s="8" t="n">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>50038</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>MLA2090592693</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Proteína Isolada Hidrolizada Gold Nutrition 2lb Chocolate Gourmet Milk Chocolate</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>45592.51</v>
+      </c>
+      <c r="E99" s="8" t="n">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>50043</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>MLA2123719629</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato Micronizada Gold Nutrition 300g Neutro Sin Sabor</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>11113.17</v>
+      </c>
+      <c r="E100" s="8" t="n">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>50043</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>MLA2123746311</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Creatina Monohidrato Micronizada Gold Nutrition 300g Neutro Sin Sabor</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>11113.17</v>
+      </c>
+      <c r="E101" s="8" t="n">
+        <v>46300</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>50039</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MLA2090594293</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Whey Protein Gold Nutrition 2 Libras Proteína 100% Vainilla Gourmet</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>36636.84</v>
+      </c>
+      <c r="E102" s="8" t="n">
         <v>46300</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corregir costos 50038/50039/50043: son +IVA (netos), sin dividir por 1,21; regla de IVA en CLAUDE.md
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B6Ej9HH2pZG2xD9hqQfC1p
</commit_message>
<xml_diff>
--- a/data/Costos.xlsx
+++ b/data/Costos.xlsx
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="D96" s="0" t="n">
-        <v>45592.51</v>
+        <v>55166.94</v>
       </c>
       <c r="E96" s="8" t="n">
         <v>46300</v>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="D97" s="0" t="n">
-        <v>36636.84</v>
+        <v>44330.58</v>
       </c>
       <c r="E97" s="8" t="n">
         <v>46300</v>
@@ -2414,91 +2414,91 @@
         </is>
       </c>
       <c r="D98" s="0" t="n">
-        <v>11113.17</v>
+        <v>13446.94</v>
       </c>
       <c r="E98" s="8" t="n">
         <v>46300</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="n">
+      <c r="A99" s="0" t="n">
         <v>50038</v>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="0" t="inlineStr">
         <is>
           <t>MLA2090592693</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="0" t="inlineStr">
         <is>
           <t>Proteína Isolada Hidrolizada Gold Nutrition 2lb Chocolate Gourmet Milk Chocolate</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v>45592.51</v>
+      <c r="D99" s="0" t="n">
+        <v>55166.94</v>
       </c>
       <c r="E99" s="8" t="n">
         <v>46300</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="n">
+      <c r="A100" s="0" t="n">
         <v>50043</v>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B100" s="0" t="inlineStr">
         <is>
           <t>MLA2123719629</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C100" s="0" t="inlineStr">
         <is>
           <t>Creatina Monohidrato Micronizada Gold Nutrition 300g Neutro Sin Sabor</t>
         </is>
       </c>
-      <c r="D100" t="n">
-        <v>11113.17</v>
+      <c r="D100" s="0" t="n">
+        <v>13446.94</v>
       </c>
       <c r="E100" s="8" t="n">
         <v>46300</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="n">
+      <c r="A101" s="0" t="n">
         <v>50043</v>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="0" t="inlineStr">
         <is>
           <t>MLA2123746311</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="0" t="inlineStr">
         <is>
           <t>Creatina Monohidrato Micronizada Gold Nutrition 300g Neutro Sin Sabor</t>
         </is>
       </c>
-      <c r="D101" t="n">
-        <v>11113.17</v>
+      <c r="D101" s="0" t="n">
+        <v>13446.94</v>
       </c>
       <c r="E101" s="8" t="n">
         <v>46300</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="n">
+      <c r="A102" s="0" t="n">
         <v>50039</v>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B102" s="0" t="inlineStr">
         <is>
           <t>MLA2090594293</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="0" t="inlineStr">
         <is>
           <t>Whey Protein Gold Nutrition 2 Libras Proteína 100% Vainilla Gourmet</t>
         </is>
       </c>
-      <c r="D102" t="n">
-        <v>36636.84</v>
+      <c r="D102" s="0" t="n">
+        <v>44330.58</v>
       </c>
       <c r="E102" s="8" t="n">
         <v>46300</v>

</xml_diff>